<commit_message>
modifications for lab meeting
</commit_message>
<xml_diff>
--- a/data/plant_codes.xlsx
+++ b/data/plant_codes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sierrajech/Desktop/NAU_DIRT/Projects/Faist_seedbanks/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15B8DFBA-A2DB-6C47-8B7E-5528740A7896}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F27DA6E-5E90-7E4D-9236-B0781516B9B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="660" windowWidth="16680" windowHeight="10080" xr2:uid="{32686EA9-2D8F-164B-BD73-057F9D52E9B5}"/>
+    <workbookView xWindow="380" yWindow="660" windowWidth="21680" windowHeight="9740" xr2:uid="{32686EA9-2D8F-164B-BD73-057F9D52E9B5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="42">
   <si>
     <t>monocot_dicot</t>
   </si>
@@ -147,6 +147,21 @@
   </si>
   <si>
     <t>greenhouse weed</t>
+  </si>
+  <si>
+    <t>lifespan</t>
+  </si>
+  <si>
+    <t>annual</t>
+  </si>
+  <si>
+    <t>perennial</t>
+  </si>
+  <si>
+    <t>season</t>
+  </si>
+  <si>
+    <t>cool</t>
   </si>
 </sst>
 </file>
@@ -527,19 +542,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75AC54EB-47CD-D94C-8AE7-03C851827858}">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="12.6640625" customWidth="1"/>
+    <col min="10" max="10" width="17" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -556,25 +572,31 @@
         <v>5</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -591,22 +613,28 @@
         <v>17</v>
       </c>
       <c r="F2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H2" t="s">
         <v>25</v>
       </c>
-      <c r="G2" t="s">
+      <c r="I2" t="s">
         <v>27</v>
-      </c>
-      <c r="H2" t="s">
-        <v>26</v>
-      </c>
-      <c r="I2">
-        <v>7.4999999999999997E-2</v>
       </c>
       <c r="J2" t="s">
         <v>26</v>
       </c>
+      <c r="K2">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="L2" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -623,22 +651,28 @@
         <v>18</v>
       </c>
       <c r="F3" t="s">
+        <v>38</v>
+      </c>
+      <c r="G3" t="s">
+        <v>41</v>
+      </c>
+      <c r="H3" t="s">
         <v>25</v>
       </c>
-      <c r="G3" t="s">
+      <c r="I3" t="s">
         <v>27</v>
-      </c>
-      <c r="H3" t="s">
-        <v>26</v>
-      </c>
-      <c r="I3">
-        <v>0.03</v>
       </c>
       <c r="J3" t="s">
         <v>26</v>
       </c>
+      <c r="K3">
+        <v>0.03</v>
+      </c>
+      <c r="L3" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>31</v>
       </c>
@@ -655,19 +689,25 @@
         <v>34</v>
       </c>
       <c r="F4" t="s">
+        <v>39</v>
+      </c>
+      <c r="G4" t="s">
+        <v>41</v>
+      </c>
+      <c r="H4" t="s">
         <v>35</v>
       </c>
-      <c r="G4" t="s">
+      <c r="I4" t="s">
         <v>27</v>
       </c>
-      <c r="H4" t="s">
+      <c r="J4" t="s">
         <v>26</v>
       </c>
-      <c r="K4" t="s">
+      <c r="M4" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -684,22 +724,28 @@
         <v>19</v>
       </c>
       <c r="F5" t="s">
+        <v>38</v>
+      </c>
+      <c r="G5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H5" t="s">
         <v>35</v>
       </c>
-      <c r="G5" t="s">
+      <c r="I5" t="s">
         <v>28</v>
       </c>
-      <c r="H5" t="s">
+      <c r="J5" t="s">
         <v>26</v>
       </c>
-      <c r="I5">
+      <c r="K5">
         <v>3</v>
       </c>
-      <c r="J5" t="s">
+      <c r="L5" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -716,18 +762,24 @@
         <v>24</v>
       </c>
       <c r="F6" t="s">
+        <v>39</v>
+      </c>
+      <c r="G6" t="s">
+        <v>41</v>
+      </c>
+      <c r="H6" t="s">
         <v>25</v>
       </c>
-      <c r="G6" t="s">
+      <c r="I6" t="s">
         <v>28</v>
       </c>
-      <c r="H6" t="s">
+      <c r="J6" t="s">
         <v>26</v>
       </c>
-      <c r="I6">
+      <c r="K6">
         <v>0.1</v>
       </c>
-      <c r="J6" t="s">
+      <c r="L6" t="s">
         <v>26</v>
       </c>
     </row>

</xml_diff>